<commit_message>
Python Code and updated Menu
</commit_message>
<xml_diff>
--- a/Menu.xlsx
+++ b/Menu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43ACD0CF-4CF7-4DC2-875C-2A9507DD21FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8373CE-7C81-4889-B93B-6EF6C8A6D987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8F099DAA-0706-44C8-A923-6852E9A1E4AD}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
   <si>
     <t>Item Name</t>
   </si>
@@ -115,25 +115,64 @@
   </si>
   <si>
     <t>Hot Fudge Sundae</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Snack</t>
+  </si>
+  <si>
+    <t>Beverage</t>
+  </si>
+  <si>
+    <t>Dessert</t>
+  </si>
+  <si>
+    <t>Chocolate Shake</t>
+  </si>
+  <si>
+    <t>Iced Tea</t>
+  </si>
+  <si>
+    <t>Caramel Sundae</t>
+  </si>
+  <si>
+    <t>Apple Pie</t>
+  </si>
+  <si>
+    <t>Bottled Water</t>
+  </si>
+  <si>
+    <t>Extra Cheese</t>
+  </si>
+  <si>
+    <t>Add-on</t>
+  </si>
+  <si>
+    <t>Extra Tomato</t>
+  </si>
+  <si>
+    <t>Extra Lettuce</t>
+  </si>
+  <si>
+    <t>Extra Olives</t>
+  </si>
+  <si>
+    <t>Extra Onions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -144,7 +183,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -152,33 +191,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -493,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB324BDC-5C53-408C-A36E-5E81D26D052B}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.109375" customWidth="1"/>
@@ -503,489 +521,813 @@
     <col min="5" max="5" width="19.33203125" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
     <col min="7" max="7" width="19.77734375" customWidth="1"/>
+    <col min="8" max="8" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2">
         <v>120</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2">
         <v>35</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2">
         <v>45</v>
       </c>
-      <c r="F2" s="2">
+      <c r="G2">
         <v>75</v>
       </c>
-      <c r="G2" s="2">
+      <c r="H2">
         <v>4500</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3">
         <v>135</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3">
         <v>50</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3">
         <v>12</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3">
         <v>62</v>
       </c>
-      <c r="F3" s="2">
+      <c r="G3">
         <v>73</v>
       </c>
-      <c r="G3" s="2">
+      <c r="H3">
         <v>4200</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4">
         <v>210</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D4">
         <v>75</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E4">
         <v>20</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4">
         <v>95</v>
       </c>
-      <c r="F4" s="2">
+      <c r="G4">
         <v>115</v>
       </c>
-      <c r="G4" s="2">
+      <c r="H4">
         <v>1200</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="54" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5">
         <v>235</v>
       </c>
-      <c r="C5" s="2">
+      <c r="D5">
         <v>95</v>
       </c>
-      <c r="D5" s="2">
+      <c r="E5">
         <v>22</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5">
         <v>117</v>
       </c>
-      <c r="F5" s="2">
+      <c r="G5">
         <v>118</v>
       </c>
-      <c r="G5" s="2">
+      <c r="H5">
         <v>1500</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6">
         <v>110</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D6">
         <v>18</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E6">
         <v>15</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6">
         <v>33</v>
       </c>
-      <c r="F6" s="2">
+      <c r="G6">
         <v>77</v>
       </c>
-      <c r="G6" s="2">
+      <c r="H6">
         <v>6000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7">
         <v>170</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7">
         <v>65</v>
       </c>
-      <c r="D7" s="2">
+      <c r="E7">
         <v>15</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7">
         <v>80</v>
       </c>
-      <c r="F7" s="2">
+      <c r="G7">
         <v>90</v>
       </c>
-      <c r="G7" s="2">
+      <c r="H7">
         <v>2100</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
         <v>55</v>
       </c>
-      <c r="C8" s="2">
+      <c r="D8">
         <v>15</v>
       </c>
-      <c r="D8" s="2">
+      <c r="E8">
         <v>8</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8">
         <v>23</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8">
         <v>32</v>
       </c>
-      <c r="G8" s="2">
+      <c r="H8">
         <v>3800</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9">
         <v>70</v>
       </c>
-      <c r="C9" s="2">
+      <c r="D9">
         <v>20</v>
       </c>
-      <c r="D9" s="2">
+      <c r="E9">
         <v>10</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9">
         <v>30</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9">
         <v>40</v>
       </c>
-      <c r="G9" s="2">
+      <c r="H9">
         <v>7200</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10">
         <v>90</v>
       </c>
-      <c r="C10" s="2">
+      <c r="D10">
         <v>8</v>
       </c>
-      <c r="D10" s="2">
+      <c r="E10">
         <v>2</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10">
         <v>10</v>
       </c>
-      <c r="F10" s="2">
+      <c r="G10">
         <v>80</v>
       </c>
-      <c r="G10" s="2">
+      <c r="H10">
         <v>8500</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11">
         <v>130</v>
       </c>
-      <c r="C11" s="2">
+      <c r="D11">
         <v>30</v>
       </c>
-      <c r="D11" s="2">
+      <c r="E11">
         <v>15</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11">
         <v>45</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G11">
         <v>85</v>
       </c>
-      <c r="G11" s="2">
+      <c r="H11">
         <v>2800</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12">
         <v>35</v>
       </c>
-      <c r="C12" s="2">
+      <c r="D12">
         <v>8</v>
       </c>
-      <c r="D12" s="2">
+      <c r="E12">
         <v>5</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12">
         <v>13</v>
       </c>
-      <c r="F12" s="2">
+      <c r="G12">
         <v>22</v>
       </c>
-      <c r="G12" s="2">
+      <c r="H12">
         <v>5000</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13">
         <v>115</v>
       </c>
-      <c r="C13" s="2">
+      <c r="D13">
         <v>40</v>
       </c>
-      <c r="D13" s="2">
+      <c r="E13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13">
         <v>50</v>
       </c>
-      <c r="F13" s="2">
+      <c r="G13">
         <v>65</v>
       </c>
-      <c r="G13" s="2">
+      <c r="H13">
         <v>1900</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14">
         <v>165</v>
       </c>
-      <c r="C14" s="2">
+      <c r="D14">
         <v>85</v>
       </c>
-      <c r="D14" s="2">
+      <c r="E14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14">
         <v>100</v>
       </c>
-      <c r="F14" s="2">
+      <c r="G14">
         <v>65</v>
       </c>
-      <c r="G14" s="2">
+      <c r="H14">
         <v>800</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15">
         <v>140</v>
       </c>
-      <c r="C15" s="2">
+      <c r="D15">
         <v>70</v>
       </c>
-      <c r="D15" s="2">
+      <c r="E15">
         <v>18</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15">
         <v>88</v>
       </c>
-      <c r="F15" s="2">
+      <c r="G15">
         <v>52</v>
       </c>
-      <c r="G15" s="2">
+      <c r="H15">
         <v>1100</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16">
         <v>100</v>
       </c>
-      <c r="C16" s="2">
+      <c r="D16">
         <v>30</v>
       </c>
-      <c r="D16" s="2">
+      <c r="E16">
         <v>12</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16">
         <v>42</v>
       </c>
-      <c r="F16" s="2">
+      <c r="G16">
         <v>58</v>
       </c>
-      <c r="G16" s="2">
+      <c r="H16">
         <v>900</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
         <v>110</v>
       </c>
-      <c r="C17" s="2">
+      <c r="D17">
         <v>35</v>
       </c>
-      <c r="D17" s="2">
+      <c r="E17">
         <v>12</v>
       </c>
-      <c r="E17" s="2">
+      <c r="F17">
         <v>47</v>
       </c>
-      <c r="F17" s="2">
+      <c r="G17">
         <v>63</v>
       </c>
-      <c r="G17" s="2">
+      <c r="H17">
         <v>1150</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18">
         <v>50</v>
       </c>
-      <c r="C18" s="2">
+      <c r="D18">
         <v>12</v>
       </c>
-      <c r="D18" s="2">
+      <c r="E18">
         <v>10</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18">
         <v>22</v>
       </c>
-      <c r="F18" s="2">
-        <v>28</v>
-      </c>
-      <c r="G18" s="2">
+      <c r="G18">
+        <v>28</v>
+      </c>
+      <c r="H18">
         <v>2400</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>24</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19">
         <v>180</v>
       </c>
-      <c r="C19" s="2">
+      <c r="D19">
         <v>65</v>
       </c>
-      <c r="D19" s="2">
+      <c r="E19">
         <v>18</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19">
         <v>83</v>
       </c>
-      <c r="F19" s="2">
+      <c r="G19">
         <v>97</v>
       </c>
-      <c r="G19" s="2">
+      <c r="H19">
         <v>700</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
         <v>210</v>
       </c>
-      <c r="C20" s="2">
+      <c r="D20">
         <v>85</v>
       </c>
-      <c r="D20" s="2">
+      <c r="E20">
         <v>20</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20">
         <v>105</v>
       </c>
-      <c r="F20" s="2">
+      <c r="G20">
         <v>105</v>
       </c>
-      <c r="G20" s="2">
+      <c r="H20">
         <v>950</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="40.799999999999997" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21">
         <v>105</v>
       </c>
-      <c r="C21" s="2">
+      <c r="D21">
         <v>35</v>
       </c>
-      <c r="D21" s="2">
+      <c r="E21">
         <v>5</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21">
         <v>40</v>
       </c>
-      <c r="F21" s="2">
+      <c r="G21">
         <v>65</v>
       </c>
-      <c r="G21" s="2">
+      <c r="H21">
         <v>2300</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22">
+        <v>140</v>
+      </c>
+      <c r="D22">
+        <v>40</v>
+      </c>
+      <c r="E22">
+        <v>10</v>
+      </c>
+      <c r="F22">
+        <v>50</v>
+      </c>
+      <c r="G22">
+        <v>90</v>
+      </c>
+      <c r="H22">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23">
+        <v>70</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23">
+        <v>25</v>
+      </c>
+      <c r="G23">
+        <v>45</v>
+      </c>
+      <c r="H23">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24">
+        <v>120</v>
+      </c>
+      <c r="D24">
+        <v>30</v>
+      </c>
+      <c r="E24">
+        <v>10</v>
+      </c>
+      <c r="F24">
+        <v>40</v>
+      </c>
+      <c r="G24">
+        <v>80</v>
+      </c>
+      <c r="H24">
+        <v>2800</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25">
+        <v>90</v>
+      </c>
+      <c r="D25">
+        <v>30</v>
+      </c>
+      <c r="E25">
+        <v>10</v>
+      </c>
+      <c r="F25">
+        <v>40</v>
+      </c>
+      <c r="G25">
+        <v>50</v>
+      </c>
+      <c r="H25">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26">
+        <v>40</v>
+      </c>
+      <c r="D26">
+        <v>10</v>
+      </c>
+      <c r="E26">
+        <v>5</v>
+      </c>
+      <c r="F26">
+        <v>15</v>
+      </c>
+      <c r="G26">
+        <v>25</v>
+      </c>
+      <c r="H26">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27">
+        <v>25</v>
+      </c>
+      <c r="D27">
+        <v>10</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+      <c r="F27">
+        <v>12</v>
+      </c>
+      <c r="G27">
+        <v>13</v>
+      </c>
+      <c r="H27">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C28">
+        <v>15</v>
+      </c>
+      <c r="D28">
+        <v>5</v>
+      </c>
+      <c r="E28">
+        <v>2</v>
+      </c>
+      <c r="F28">
+        <v>7</v>
+      </c>
+      <c r="G28">
+        <v>8</v>
+      </c>
+      <c r="H28">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" t="s">
+        <v>37</v>
+      </c>
+      <c r="C29">
+        <v>15</v>
+      </c>
+      <c r="D29">
+        <v>5</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29">
+        <v>7</v>
+      </c>
+      <c r="G29">
+        <v>8</v>
+      </c>
+      <c r="H29">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>40</v>
+      </c>
+      <c r="B30" t="s">
+        <v>37</v>
+      </c>
+      <c r="C30">
+        <v>20</v>
+      </c>
+      <c r="D30">
+        <v>8</v>
+      </c>
+      <c r="E30">
+        <v>2</v>
+      </c>
+      <c r="F30">
+        <v>10</v>
+      </c>
+      <c r="G30">
+        <v>10</v>
+      </c>
+      <c r="H30">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31">
+        <v>10</v>
+      </c>
+      <c r="D31">
+        <v>3</v>
+      </c>
+      <c r="E31">
+        <v>2</v>
+      </c>
+      <c r="F31">
+        <v>5</v>
+      </c>
+      <c r="G31">
+        <v>5</v>
+      </c>
+      <c r="H31">
+        <v>1100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>